<commit_message>
Evolui dashboards, importação de estoques e renomeia monitoramento.
Dashboard financeira com polling em tempo real; Olho de Fabio (rotas e permissão novas com redirect legado); importação de estoque por UM e preço total com tabela de erros corrigida na preview.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/planilhas/estoques_importacao.xlsx
+++ b/planilhas/estoques_importacao.xlsx
@@ -1,53 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Estoques" sheetId="1" r:id="rId4"/>
+    <sheet name="Estoques" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="999999" calcMode="auto" fullCalcOnLoad="0" calcCompleted="1" forceFullCalc="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="4">
-  <si>
-    <t>id_cigam_unidade</t>
-  </si>
-  <si>
-    <t>id_cigam_fruta</t>
-  </si>
-  <si>
-    <t>qtd_fruta_kg</t>
-  </si>
-  <si>
-    <t>preco_medio_kg</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
+      <name val="Calibri"/>
       <strike val="0"/>
-      <u val="none"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -66,13 +45,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -362,52 +408,65 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="1" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col width="19.995" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.567" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.282" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="17.567" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID CIGAM Unidade</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ID CIGAM Fruta</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Qtd (unidade de medição)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Preço total (R$)</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>42</v>
-      </c>
-      <c r="C2">
-        <v>1500</v>
-      </c>
-      <c r="D2">
-        <v>3.25</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>000001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>000001</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <printOptions gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+  <pageSetup orientation="default" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="1" alignWithMargins="1">
     <oddHeader/>
     <oddFooter/>
     <evenHeader/>
@@ -415,6 +474,5 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>